<commit_message>
FIX: Coerce strings also in arrays. Address copilot's comments
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/LOGICAL/IF_ARRAY.xlsx
+++ b/xlsx/tests/calc_tests/LOGICAL/IF_ARRAY.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/Statistical/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B5B57C9-A83E-DB48-AA74-FBC2DD388392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E1AC6F1-C2B8-BB4B-8A3E-131451D11293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" xr2:uid="{C6CB3E91-6B53-6C4F-9CFE-9A74BA10449A}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" activeTab="1" xr2:uid="{C6CB3E91-6B53-6C4F-9CFE-9A74BA10449A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -58,6 +59,14 @@
     </bk>
   </cellMetadata>
 </metadata>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>45550</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -91,8 +100,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85030ED7-B956-0E47-81B2-A52B6E38B059}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -623,6 +633,129 @@
         <v>2</v>
       </c>
     </row>
+    <row r="20" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D20" cm="1">
+        <f t="array" ref="D20:F20">IF({TRUE,FALSE,TRUE}, {1,2,3})</f>
+        <v>1</v>
+      </c>
+      <c r="E20" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="4:6" x14ac:dyDescent="0.2">
+      <c r="D22" cm="1">
+        <f t="array" ref="D22:F22">IF({TRUE,#N/A,FALSE},1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="E22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ED1E8BC-D82E-F640-8221-D0DF26061B16}">
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" cm="1">
+        <f t="array" ref="A1:B1">YEAR({45000,46000})</f>
+        <v>2023</v>
+      </c>
+      <c r="B1">
+        <v>2025</v>
+      </c>
+      <c r="F1" cm="1">
+        <f t="array" ref="F1:F2">YEAR({"45000";"46000"})</f>
+        <v>2023</v>
+      </c>
+      <c r="H1">
+        <v>45000</v>
+      </c>
+      <c r="I1">
+        <v>46000</v>
+      </c>
+      <c r="K1" cm="1">
+        <f t="array" ref="K1:L2">DAY(H1:I2)</f>
+        <v>15</v>
+      </c>
+      <c r="L1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" cm="1">
+        <f t="array" ref="A2:B2">DAY({45000,46000})</f>
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>9</v>
+      </c>
+      <c r="F2">
+        <v>2025</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>47000</v>
+      </c>
+      <c r="K2">
+        <v>15</v>
+      </c>
+      <c r="L2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" cm="1">
+        <f t="array" ref="A3:B3">MONTH({45000,4700})</f>
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H5" cm="1">
+        <f t="array" ref="H5:I6">MONTH(H1:I2)</f>
+        <v>3</v>
+      </c>
+      <c r="I5">
+        <v>12</v>
+      </c>
+      <c r="K5" cm="1">
+        <f t="array" ref="K5:L6">YEAR(H1:I2)</f>
+        <v>2023</v>
+      </c>
+      <c r="L5">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H6">
+        <v>9</v>
+      </c>
+      <c r="I6">
+        <v>9</v>
+      </c>
+      <c r="K6">
+        <v>2024</v>
+      </c>
+      <c r="L6">
+        <v>2028</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
UPDATE: Add support for arrays in SUMIF criteria argument
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/LOGICAL/IF_ARRAY.xlsx
+++ b/xlsx/tests/calc_tests/LOGICAL/IF_ARRAY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/Statistical/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Downloads/sort/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E1AC6F1-C2B8-BB4B-8A3E-131451D11293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50741454-59AA-134E-8973-602DECE5B0C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" activeTab="1" xr2:uid="{C6CB3E91-6B53-6C4F-9CFE-9A74BA10449A}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="33600" windowHeight="18580" xr2:uid="{C6CB3E91-6B53-6C4F-9CFE-9A74BA10449A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -437,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85030ED7-B956-0E47-81B2-A52B6E38B059}">
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
@@ -633,7 +633,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="4:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D20" cm="1">
         <f t="array" ref="D20:F20">IF({TRUE,FALSE,TRUE}, {1,2,3})</f>
         <v>1</v>
@@ -645,7 +645,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="4:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="D22" cm="1">
         <f t="array" ref="D22:F22">IF({TRUE,#N/A,FALSE},1,0)</f>
         <v>1</v>
@@ -655,6 +655,43 @@
       </c>
       <c r="F22">
         <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" cm="1">
+        <f t="array" ref="A26:C26">IF({TRUE,FALSE,TRUE}, {1,2,3}, {"A"})</f>
+        <v>1</v>
+      </c>
+      <c r="B26" t="str">
+        <v>A</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" cm="1">
+        <f t="array" ref="A28:B30">IF({TRUE;FALSE;TRUE}, {1,2}, {7,8})</f>
+        <v>1</v>
+      </c>
+      <c r="B28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>7</v>
+      </c>
+      <c r="B29">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>1</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>